<commit_message>
Modificacion en Pagos Recibidos
</commit_message>
<xml_diff>
--- a/Ejemplos/EJEMPLO_rendicion_alquileres.xlsx
+++ b/Ejemplos/EJEMPLO_rendicion_alquileres.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rendición" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle por servicio" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deuda por servicio" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pagos recibidos" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -457,27 +457,26 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Rendición de alquileres</t>
+          <t>Rendición de alquileres: dinero recibido en el periodo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Periodo: 01/10/2026 al 31/10/2026  ·  Meses: Octubre 2026  ·  Emitido por: Vio</t>
+          <t>Dinero recibido del 01/10/2026 al 31/10/2026  ·  Deuda de: Octubre 2026  ·  Emitido por: Vio</t>
         </is>
       </c>
     </row>
@@ -509,40 +508,35 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Alquiler</t>
+          <t>Alquiler cobrado</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Luz</t>
+          <t>Luz cobrada</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Agua</t>
+          <t>Agua cobrada</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Total a cobrar</t>
+          <t>Total cobrado</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Pagado</t>
+          <t>Deuda pendiente</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Deuda</t>
+          <t>Aire acondicionado</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>Aire acondicionado</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Contrato</t>
         </is>
@@ -575,29 +569,26 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>33</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>667</v>
+        <v>43</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="K5" s="4" t="n">
         <v>624</v>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Alquiler · Vigente</t>
         </is>
@@ -630,29 +621,26 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>800</v>
+        <v>300</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>901</v>
+        <v>300</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>300</v>
-      </c>
-      <c r="K6" s="4" t="n">
         <v>601</v>
       </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Alquiler · Vigente</t>
         </is>
@@ -688,26 +676,23 @@
         <v>500</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>78</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>645</v>
+        <v>658</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>658</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Sí · edificio</t>
+        </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Sí · edificio</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Alquiler · Vigente</t>
         </is>
@@ -754,15 +739,12 @@
       <c r="J8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="4" t="n">
-        <v>0</v>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Anticrético · Vigente</t>
         </is>
@@ -775,21 +757,18 @@
         </is>
       </c>
       <c r="F9" s="6" t="n">
-        <v>1900</v>
+        <v>800</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>145</v>
+        <v>113</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>168</v>
+        <v>88</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>2213</v>
+        <v>1001</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>1001</v>
-      </c>
-      <c r="K9" s="6" t="n">
         <v>1225</v>
       </c>
     </row>
@@ -824,14 +803,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Detalle por servicio: a cobrar, pagado y deuda</t>
+          <t>Deuda pendiente por servicio (meses que toca el periodo, a hoy)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Periodo: 01/10/2026 al 31/10/2026  ·  Meses: Octubre 2026  ·  Emitido por: Vio</t>
+          <t>Dinero recibido del 01/10/2026 al 31/10/2026  ·  Deuda de: Octubre 2026  ·  Emitido por: Vio</t>
         </is>
       </c>
     </row>
@@ -1129,14 +1108,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Pagos recibidos (movimientos)</t>
+          <t>Pagos recibidos en el periodo (por fecha de pago)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Periodo: 01/10/2026 al 31/10/2026  ·  Meses: Octubre 2026  ·  Emitido por: Vio</t>
+          <t>Dinero recibido del 01/10/2026 al 31/10/2026  ·  Deuda de: Octubre 2026  ·  Emitido por: Vio</t>
         </is>
       </c>
     </row>

</xml_diff>